<commit_message>
changement de structure site
</commit_message>
<xml_diff>
--- a/data/Genealogie_MEME.xlsx
+++ b/data/Genealogie_MEME.xlsx
@@ -3460,145 +3460,145 @@
         <v>63</v>
       </c>
     </row>
-    <row r="34">
-      <c r="A34" s="4" t="s">
+    <row r="34" customFormat="1" s="13">
+      <c r="A34" s="14" t="s">
         <v>290</v>
       </c>
-      <c r="B34" s="4" t="s">
+      <c r="B34" s="14" t="s">
         <v>294</v>
       </c>
-      <c r="C34" s="4" t="s">
+      <c r="C34" s="14" t="s">
         <v>291</v>
       </c>
-      <c r="D34" s="4"/>
-      <c r="E34" s="4" t="s">
+      <c r="D34" s="14"/>
+      <c r="E34" s="14" t="s">
         <v>43</v>
       </c>
-      <c r="F34" s="5" t="s">
+      <c r="F34" s="15" t="s">
         <v>285</v>
       </c>
-      <c r="G34" s="4"/>
-      <c r="H34" s="5" t="s">
+      <c r="G34" s="14"/>
+      <c r="H34" s="15" t="s">
         <v>297</v>
       </c>
-      <c r="I34" s="4"/>
-      <c r="J34" s="4"/>
-      <c r="K34" s="4" t="s">
+      <c r="I34" s="14"/>
+      <c r="J34" s="14"/>
+      <c r="K34" s="14" t="s">
         <v>349</v>
       </c>
-      <c r="L34" s="4"/>
-      <c r="M34" s="4"/>
-      <c r="N34" s="4"/>
-      <c r="O34" s="4" t="s">
+      <c r="L34" s="14"/>
+      <c r="M34" s="14"/>
+      <c r="N34" s="14"/>
+      <c r="O34" s="14" t="s">
         <v>55</v>
       </c>
-      <c r="P34" s="4" t="s">
+      <c r="P34" s="14" t="s">
         <v>299</v>
       </c>
-      <c r="Q34" s="6" t="s">
+      <c r="Q34" s="16" t="s">
         <v>57</v>
       </c>
     </row>
-    <row r="35">
-      <c r="A35" s="4" t="s">
+    <row r="35" customFormat="1" s="58">
+      <c r="A35" s="59" t="s">
         <v>293</v>
       </c>
-      <c r="B35" s="4" t="s">
+      <c r="B35" s="59" t="s">
         <v>302</v>
       </c>
-      <c r="C35" s="4" t="s">
+      <c r="C35" s="59" t="s">
         <v>270</v>
       </c>
-      <c r="D35" s="4" t="s">
+      <c r="D35" s="59" t="s">
         <v>270</v>
       </c>
-      <c r="E35" s="4" t="s">
+      <c r="E35" s="59" t="s">
         <v>32</v>
       </c>
-      <c r="F35" s="5"/>
-      <c r="G35" s="4"/>
-      <c r="H35" s="5"/>
-      <c r="I35" s="4"/>
-      <c r="J35" s="4"/>
-      <c r="K35" s="4"/>
-      <c r="L35" s="4" t="s">
+      <c r="F35" s="60"/>
+      <c r="G35" s="59"/>
+      <c r="H35" s="60"/>
+      <c r="I35" s="59"/>
+      <c r="J35" s="59"/>
+      <c r="K35" s="59"/>
+      <c r="L35" s="59" t="s">
         <v>305</v>
       </c>
-      <c r="M35" s="4"/>
-      <c r="N35" s="4"/>
-      <c r="O35" s="4" t="s">
+      <c r="M35" s="59"/>
+      <c r="N35" s="59"/>
+      <c r="O35" s="59" t="s">
         <v>55</v>
       </c>
-      <c r="P35" s="4" t="s">
+      <c r="P35" s="59" t="s">
         <v>308</v>
       </c>
-      <c r="Q35" s="4"/>
-    </row>
-    <row r="36">
-      <c r="A36" s="4" t="s">
+      <c r="Q35" s="59"/>
+    </row>
+    <row r="36" customFormat="1" s="58">
+      <c r="A36" s="59" t="s">
         <v>303</v>
       </c>
-      <c r="B36" s="4" t="s">
+      <c r="B36" s="59" t="s">
         <v>89</v>
       </c>
-      <c r="C36" s="4" t="s">
+      <c r="C36" s="59" t="s">
         <v>270</v>
       </c>
-      <c r="D36" s="4" t="s">
+      <c r="D36" s="59" t="s">
         <v>270</v>
       </c>
-      <c r="E36" s="4" t="s">
+      <c r="E36" s="59" t="s">
         <v>32</v>
       </c>
-      <c r="F36" s="5"/>
-      <c r="G36" s="4"/>
-      <c r="H36" s="5"/>
-      <c r="I36" s="4"/>
-      <c r="J36" s="4"/>
-      <c r="K36" s="4"/>
-      <c r="L36" s="4" t="s">
+      <c r="F36" s="60"/>
+      <c r="G36" s="59"/>
+      <c r="H36" s="60"/>
+      <c r="I36" s="59"/>
+      <c r="J36" s="59"/>
+      <c r="K36" s="59"/>
+      <c r="L36" s="59" t="s">
         <v>304</v>
       </c>
-      <c r="M36" s="4"/>
-      <c r="N36" s="4"/>
-      <c r="O36" s="4" t="s">
+      <c r="M36" s="59"/>
+      <c r="N36" s="59"/>
+      <c r="O36" s="59" t="s">
         <v>55</v>
       </c>
-      <c r="P36" s="4" t="s">
+      <c r="P36" s="59" t="s">
         <v>308</v>
       </c>
-      <c r="Q36" s="4"/>
-    </row>
-    <row r="37" customFormat="1" s="58">
-      <c r="A37" s="59" t="s">
+      <c r="Q36" s="59"/>
+    </row>
+    <row r="37" customFormat="1" s="43">
+      <c r="A37" s="44" t="s">
         <v>309</v>
       </c>
-      <c r="B37" s="59" t="s">
+      <c r="B37" s="44" t="s">
         <v>310</v>
       </c>
-      <c r="C37" s="59" t="s">
+      <c r="C37" s="44" t="s">
         <v>65</v>
       </c>
-      <c r="D37" s="59"/>
-      <c r="E37" s="59" t="s">
+      <c r="D37" s="44"/>
+      <c r="E37" s="44" t="s">
         <v>43</v>
       </c>
-      <c r="F37" s="60"/>
-      <c r="G37" s="59"/>
-      <c r="H37" s="60"/>
-      <c r="I37" s="59"/>
-      <c r="J37" s="59"/>
-      <c r="K37" s="59"/>
-      <c r="L37" s="59"/>
-      <c r="M37" s="59"/>
-      <c r="N37" s="59"/>
-      <c r="O37" s="59" t="s">
+      <c r="F37" s="45"/>
+      <c r="G37" s="44"/>
+      <c r="H37" s="45"/>
+      <c r="I37" s="44"/>
+      <c r="J37" s="44"/>
+      <c r="K37" s="44"/>
+      <c r="L37" s="44"/>
+      <c r="M37" s="44"/>
+      <c r="N37" s="44"/>
+      <c r="O37" s="44" t="s">
         <v>55</v>
       </c>
-      <c r="P37" s="59" t="s">
+      <c r="P37" s="44" t="s">
         <v>313</v>
       </c>
-      <c r="Q37" s="59"/>
+      <c r="Q37" s="44"/>
     </row>
     <row r="38">
       <c r="A38" s="4" t="s">

</xml_diff>